<commit_message>
Successfully ran RPA CRNs with 6 species and 8 reactions. Still testing the 2 species case.
</commit_message>
<xml_diff>
--- a/apps_results_MAK_REINFORCE/RPA_2species_2rxns/RPA_2species_2rxns_MAK_REINFORCE.xlsx
+++ b/apps_results_MAK_REINFORCE/RPA_2species_2rxns/RPA_2species_2rxns_MAK_REINFORCE.xlsx
@@ -10,14 +10,14 @@
     <sheet r:id="rId1" sheetId="1" name="Data"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">=Data!$A$1:$W$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$W$5</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
   <si>
     <t>Timestamp</t>
   </si>
@@ -88,18 +88,15 @@
     <t>Structure Head Temperature</t>
   </si>
   <si>
-    <t>2025-11-21 22:20:07</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/36853114bef94d1eaa5f1dc1dbc31a8a</t>
+    <t>2025-11-24 13:20:39</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/0d172f74c1f846f4862e5da34a046690</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Zombie topology discovered.</t>
-  </si>
-  <si>
     <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
@@ -118,16 +115,37 @@
     <t>{'target_entropy_ratio_to_max': np.float64(0.4686790650623293), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
   </si>
   <si>
-    <t>2025-11-21 23:05:10</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/28335e8641354096bb32bc98b6489163</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Put much more weight on the structure head entropy to push it to discover other topologies (if they exist). Another topology (trivially different) is obtained. </t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 100.0, 'entropy_weight_continuous_head': 0.01, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+    <t>2025-11-24 13:48:21</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/a84a44403ca8445db5278ac51b81ab80</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 10.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-11-24 15:21:22</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/fb46dde70f234806afaf7d6b406c539f</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 5.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-11-24 15:53:06</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/d0e8b0318dbf49958a67223aa5308aa7</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 8.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
 </sst>
 </file>
@@ -145,13 +163,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -183,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -193,6 +211,9 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -502,35 +523,35 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="139.57642857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="257.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="4" width="74.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="4" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="4" width="133.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="11.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="255.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="74.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="133.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -601,7 +622,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
@@ -611,97 +632,85 @@
       <c r="C2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="3">
+        <v>200</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="2">
-        <v>300</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="3">
+        <v>5</v>
+      </c>
+      <c r="L2" s="3">
+        <v>1024</v>
+      </c>
+      <c r="M2" s="3">
+        <v>10240</v>
+      </c>
+      <c r="N2" s="3">
+        <v>128</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="2">
-        <v>5</v>
-      </c>
-      <c r="L2" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M2" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N2" s="2">
-        <v>128</v>
-      </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="3">
         <v>30</v>
       </c>
-      <c r="P2" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q2" s="2">
+      <c r="R2" s="3">
+        <v>100</v>
+      </c>
+      <c r="S2" s="3">
+        <v>1000</v>
+      </c>
+      <c r="T2" s="3">
+        <v>1</v>
+      </c>
+      <c r="U2" s="3">
+        <v>9</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R2" s="2">
-        <v>100</v>
-      </c>
-      <c r="S2" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T2" s="2">
-        <v>1</v>
-      </c>
-      <c r="U2" s="2">
-        <v>9</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="W2" s="1" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="H3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="3">
+        <v>200</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="I3" s="3">
-        <v>300</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="K3" s="3">
         <v>5</v>
@@ -716,7 +725,7 @@
         <v>128</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P3" s="3">
         <v>10</v>
@@ -737,10 +746,140 @@
         <v>9</v>
       </c>
       <c r="V3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="W3" s="1" t="s">
-        <v>32</v>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+      <c r="A4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="2">
+        <v>200</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="2">
+        <v>5</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M4" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N4" s="2">
+        <v>128</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>30</v>
+      </c>
+      <c r="R4" s="2">
+        <v>100</v>
+      </c>
+      <c r="S4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T4" s="2">
+        <v>1</v>
+      </c>
+      <c r="U4" s="2">
+        <v>9</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+      <c r="A5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="2">
+        <v>200</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" s="2">
+        <v>5</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M5" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N5" s="2">
+        <v>128</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>30</v>
+      </c>
+      <c r="R5" s="2">
+        <v>100</v>
+      </c>
+      <c r="S5" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T5" s="2">
+        <v>1</v>
+      </c>
+      <c r="U5" s="2">
+        <v>9</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stylistic changes and succesfull plotting results for oscillators. Still working on oscillators with frequency tuning.
</commit_message>
<xml_diff>
--- a/apps_results_MAK_REINFORCE/RPA_2species_2rxns/RPA_2species_2rxns_MAK_REINFORCE.xlsx
+++ b/apps_results_MAK_REINFORCE/RPA_2species_2rxns/RPA_2species_2rxns_MAK_REINFORCE.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Timestamp</t>
   </si>
@@ -94,7 +94,7 @@
     <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/0d172f74c1f846f4862e5da34a046690</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t/>
   </si>
   <si>
     <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
@@ -121,9 +121,6 @@
     <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/a84a44403ca8445db5278ac51b81ab80</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 10.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
@@ -140,9 +137,6 @@
   </si>
   <si>
     <t>https://www.comet.com/maurice-filo/rpa-2species-2rxns-mak-reinforce/d0e8b0318dbf49958a67223aa5308aa7</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 8.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
@@ -153,19 +147,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -201,15 +189,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
@@ -526,32 +511,32 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="255.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="74.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="6" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="6" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="6" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="5" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="5" width="133.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="11.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="255.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="74.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="4" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="4" width="133.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -629,7 +614,7 @@
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D2" s="1"/>
@@ -641,43 +626,43 @@
       <c r="H2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="2">
         <v>200</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="2">
         <v>5</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="2">
         <v>1024</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2" s="2">
         <v>10240</v>
       </c>
-      <c r="N2" s="3">
+      <c r="N2" s="2">
         <v>128</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="3">
+      <c r="P2" s="2">
         <v>10</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="Q2" s="2">
         <v>30</v>
       </c>
-      <c r="R2" s="3">
+      <c r="R2" s="2">
         <v>100</v>
       </c>
-      <c r="S2" s="3">
+      <c r="S2" s="2">
         <v>1000</v>
       </c>
-      <c r="T2" s="3">
+      <c r="T2" s="2">
         <v>1</v>
       </c>
-      <c r="U2" s="3">
+      <c r="U2" s="2">
         <v>9</v>
       </c>
       <c r="V2" s="1" t="s">
@@ -694,55 +679,55 @@
       <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>34</v>
+      <c r="C3" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="2">
         <v>200</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="2">
         <v>5</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="2">
         <v>1024</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="2">
         <v>10240</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="2">
         <v>128</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P3" s="3">
+      <c r="P3" s="2">
         <v>10</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="Q3" s="2">
         <v>30</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="2">
         <v>100</v>
       </c>
-      <c r="S3" s="3">
+      <c r="S3" s="2">
         <v>1000</v>
       </c>
-      <c r="T3" s="3">
+      <c r="T3" s="2">
         <v>1</v>
       </c>
-      <c r="U3" s="3">
+      <c r="U3" s="2">
         <v>9</v>
       </c>
       <c r="V3" s="1" t="s">
@@ -752,21 +737,21 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>27</v>
@@ -817,21 +802,19 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>27</v>

</xml_diff>